<commit_message>
fix(mapa): soporte universal para SI, SÍ, minúsculas y checkboxes en fórmulas de correlatividades
</commit_message>
<xml_diff>
--- a/data/mapas/Mapa_de_Carrera_Filosofia.xlsx
+++ b/data/mapas/Mapa_de_Carrera_Filosofia.xlsx
@@ -579,9 +579,9 @@
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
@@ -608,12 +608,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>¿Cursada Regular? (SÍ / NO)</t>
+          <t>¿Cursada Regular? (SI / NO)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>¿Final Aprobado? (SÍ / NO)</t>
+          <t>¿Final Aprobado? (SI / NO)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -679,15 +679,15 @@
         </is>
       </c>
       <c r="E5" s="9">
-        <f>IF(B5="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B5="SI",B5="SÍ",B5=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F5" s="9">
-        <f>IF(C5="SÍ","APROBADA",IF(B5="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C5="SI",C5="SÍ",C5=TRUE),"APROBADA",IF(OR(B5="SI",B5="SÍ",B5=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G5" s="9">
-        <f>IF(C5="SÍ","✅ Materia Aprobada",IF(B5="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C5="SI",C5="SÍ",C5=TRUE),"✅ Materia Aprobada",IF(OR(B5="SI",B5="SÍ",B5=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="J5" s="7">
-        <f>COUNTIF(B4:B50, "SÍ")</f>
+        <f>COUNTIF(B4:B50, "S*") + COUNTIF(B4:B50, TRUE)</f>
         <v/>
       </c>
     </row>
@@ -722,15 +722,15 @@
         </is>
       </c>
       <c r="E6" s="9">
-        <f>IF(B6="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B6="SI",B6="SÍ",B6=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>IF(C6="SÍ","APROBADA",IF(B6="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C6="SI",C6="SÍ",C6=TRUE),"APROBADA",IF(OR(B6="SI",B6="SÍ",B6=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G6" s="9">
-        <f>IF(C6="SÍ","✅ Materia Aprobada",IF(B6="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C6="SI",C6="SÍ",C6=TRUE),"✅ Materia Aprobada",IF(OR(B6="SI",B6="SÍ",B6=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="J6" s="7">
-        <f>COUNTIF(C4:C50, "SÍ")</f>
+        <f>COUNTIF(C4:C50, "S*") + COUNTIF(C4:C50, TRUE)</f>
         <v/>
       </c>
     </row>
@@ -765,15 +765,15 @@
         </is>
       </c>
       <c r="E7" s="9">
-        <f>IF(B7="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B7="SI",B7="SÍ",B7=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>IF(C7="SÍ","APROBADA",IF(B7="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C7="SI",C7="SÍ",C7=TRUE),"APROBADA",IF(OR(B7="SI",B7="SÍ",B7=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>IF(C7="SÍ","✅ Materia Aprobada",IF(B7="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C7="SI",C7="SÍ",C7=TRUE),"✅ Materia Aprobada",IF(OR(B7="SI",B7="SÍ",B7=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="J7" s="7">
-        <f>COUNTIF(B4:B50, "SÍ") - COUNTIF(C4:C50, "SÍ")</f>
+        <f>J5-J6</f>
         <v/>
       </c>
     </row>
@@ -808,15 +808,15 @@
         </is>
       </c>
       <c r="E8" s="9">
-        <f>IF(B8="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B8="SI",B8="SÍ",B8=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>IF(C8="SÍ","APROBADA",IF(B8="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C8="SI",C8="SÍ",C8=TRUE),"APROBADA",IF(OR(B8="SI",B8="SÍ",B8=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>IF(C8="SÍ","✅ Materia Aprobada",IF(B8="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C8="SI",C8="SÍ",C8=TRUE),"✅ Materia Aprobada",IF(OR(B8="SI",B8="SÍ",B8=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="J8" s="13">
-        <f>COUNTIF(B4:B50, "SÍ") / 42</f>
+        <f>J5/42</f>
         <v/>
       </c>
     </row>
@@ -851,15 +851,15 @@
         </is>
       </c>
       <c r="E9" s="9">
-        <f>IF(B9="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B9="SI",B9="SÍ",B9=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>IF(C9="SÍ","APROBADA",IF(B9="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C9="SI",C9="SÍ",C9=TRUE),"APROBADA",IF(OR(B9="SI",B9="SÍ",B9=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>IF(C9="SÍ","✅ Materia Aprobada",IF(B9="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C9="SI",C9="SÍ",C9=TRUE),"✅ Materia Aprobada",IF(OR(B9="SI",B9="SÍ",B9=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="J9" s="13">
-        <f>COUNTIF(C4:C50, "SÍ") / 42</f>
+        <f>J6/42</f>
         <v/>
       </c>
     </row>
@@ -894,15 +894,15 @@
         </is>
       </c>
       <c r="E10" s="9">
-        <f>IF(B10="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B10="SI",B10="SÍ",B10=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>IF(C10="SÍ","APROBADA",IF(B10="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C10="SI",C10="SÍ",C10=TRUE),"APROBADA",IF(OR(B10="SI",B10="SÍ",B10=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G10" s="9">
-        <f>IF(C10="SÍ","✅ Materia Aprobada",IF(B10="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C10="SI",C10="SÍ",C10=TRUE),"✅ Materia Aprobada",IF(OR(B10="SI",B10="SÍ",B10=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -928,15 +928,15 @@
         </is>
       </c>
       <c r="E11" s="9">
-        <f>IF(B11="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B11="SI",B11="SÍ",B11=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F11" s="9">
-        <f>IF(C11="SÍ","APROBADA",IF(B11="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C11="SI",C11="SÍ",C11=TRUE),"APROBADA",IF(OR(B11="SI",B11="SÍ",B11=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G11" s="9">
-        <f>IF(C11="SÍ","✅ Materia Aprobada",IF(B11="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C11="SI",C11="SÍ",C11=TRUE),"✅ Materia Aprobada",IF(OR(B11="SI",B11="SÍ",B11=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I11" s="14" t="inlineStr">
@@ -967,20 +967,20 @@
         </is>
       </c>
       <c r="E12" s="9">
-        <f>IF(B12="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B12="SI",B12="SÍ",B12=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>IF(C12="SÍ","APROBADA",IF(B12="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C12="SI",C12="SÍ",C12=TRUE),"APROBADA",IF(OR(B12="SI",B12="SÍ",B12=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G12" s="9">
-        <f>IF(C12="SÍ","✅ Materia Aprobada",IF(B12="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C12="SI",C12="SÍ",C12=TRUE),"✅ Materia Aprobada",IF(OR(B12="SI",B12="SÍ",B12=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
-          <t>1. Escribí 'SÍ' en la columna B cuando tengas la cursada regular aprobada.</t>
+          <t>1. Seleccioná 'SI' o 'SÍ' en la columna B cuando tengas la cursada regular aprobada.</t>
         </is>
       </c>
     </row>
@@ -1006,20 +1006,20 @@
         </is>
       </c>
       <c r="E13" s="9">
-        <f>IF(B13="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B13="SI",B13="SÍ",B13=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>IF(C13="SÍ","APROBADA",IF(B13="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C13="SI",C13="SÍ",C13=TRUE),"APROBADA",IF(OR(B13="SI",B13="SÍ",B13=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G13" s="9">
-        <f>IF(C13="SÍ","✅ Materia Aprobada",IF(B13="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C13="SI",C13="SÍ",C13=TRUE),"✅ Materia Aprobada",IF(OR(B13="SI",B13="SÍ",B13=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>2. Escribí 'SÍ' en la columna C cuando hayas aprobado el examen final.</t>
+          <t>2. Seleccioná 'SI' o 'SÍ' en la columna C cuando hayas aprobado el examen final.</t>
         </is>
       </c>
     </row>
@@ -1045,15 +1045,15 @@
         </is>
       </c>
       <c r="E14" s="9">
-        <f>IF(B14="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B14="SI",B14="SÍ",B14=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>IF(C14="SÍ","APROBADA",IF(B14="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C14="SI",C14="SÍ",C14=TRUE),"APROBADA",IF(OR(B14="SI",B14="SÍ",B14=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>IF(C14="SÍ","✅ Materia Aprobada",IF(B14="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C14="SI",C14="SÍ",C14=TRUE),"✅ Materia Aprobada",IF(OR(B14="SI",B14="SÍ",B14=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I14" s="15" t="inlineStr">
@@ -1096,15 +1096,15 @@
         </is>
       </c>
       <c r="E16" s="9">
-        <f>IF(B16="SÍ","CURSADA REGULAR",IF(AND(B10="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B16="SI",B16="SÍ",B16=TRUE),"CURSADA REGULAR",IF(AND(OR(B10="SI",B10="SÍ",B10=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>IF(C16="SÍ","APROBADA",IF(AND(B16="SÍ",AND(C10="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C16="SI",C16="SÍ",C16=TRUE),"APROBADA",IF(AND(OR(B16="SI",B16="SÍ",B16=TRUE),AND(OR(C10="SI",C10="SÍ",C10=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G16" s="9">
-        <f>IF(C16="SÍ","✅ Materia Aprobada",IF(B16="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C16="SI",C16="SÍ",C16=TRUE),"✅ Materia Aprobada",IF(OR(B16="SI",B16="SÍ",B16=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I16" s="15" t="inlineStr">
@@ -1135,15 +1135,15 @@
         </is>
       </c>
       <c r="E17" s="9">
-        <f>IF(B17="SÍ","CURSADA REGULAR",IF(AND(B10="SÍ",B9="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B17="SI",B17="SÍ",B17=TRUE),"CURSADA REGULAR",IF(AND(OR(B10="SI",B10="SÍ",B10=TRUE),OR(B9="SI",B9="SÍ",B9=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F17" s="9">
-        <f>IF(C17="SÍ","APROBADA",IF(AND(B17="SÍ",AND(C10="SÍ",C9="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"APROBADA",IF(AND(OR(B17="SI",B17="SÍ",B17=TRUE),AND(OR(C10="SI",C10="SÍ",C10=TRUE),OR(C9="SI",C9="SÍ",C9=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G17" s="9">
-        <f>IF(C17="SÍ","✅ Materia Aprobada",IF(B17="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"✅ Materia Aprobada",IF(OR(B17="SI",B17="SÍ",B17=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1169,15 +1169,15 @@
         </is>
       </c>
       <c r="E18" s="9">
-        <f>IF(B18="SÍ","CURSADA REGULAR",IF(AND(B6="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B18="SI",B18="SÍ",B18=TRUE),"CURSADA REGULAR",IF(AND(OR(B6="SI",B6="SÍ",B6=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>IF(C18="SÍ","APROBADA",IF(AND(B18="SÍ",AND(C6="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C18="SI",C18="SÍ",C18=TRUE),"APROBADA",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE),AND(OR(C6="SI",C6="SÍ",C6=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>IF(C18="SÍ","✅ Materia Aprobada",IF(B18="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C18="SI",C18="SÍ",C18=TRUE),"✅ Materia Aprobada",IF(OR(B18="SI",B18="SÍ",B18=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1203,15 +1203,15 @@
         </is>
       </c>
       <c r="E19" s="9">
-        <f>IF(B19="SÍ","CURSADA REGULAR",IF(AND(B6="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B19="SI",B19="SÍ",B19=TRUE),"CURSADA REGULAR",IF(AND(OR(B6="SI",B6="SÍ",B6=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F19" s="9">
-        <f>IF(C19="SÍ","APROBADA",IF(AND(B19="SÍ",AND(C6="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C19="SI",C19="SÍ",C19=TRUE),"APROBADA",IF(AND(OR(B19="SI",B19="SÍ",B19=TRUE),AND(OR(C6="SI",C6="SÍ",C6=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G19" s="9">
-        <f>IF(C19="SÍ","✅ Materia Aprobada",IF(B19="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C19="SI",C19="SÍ",C19=TRUE),"✅ Materia Aprobada",IF(OR(B19="SI",B19="SÍ",B19=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1237,15 +1237,15 @@
         </is>
       </c>
       <c r="E20" s="9">
-        <f>IF(B20="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B20="SI",B20="SÍ",B20=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>IF(C20="SÍ","APROBADA",IF(B20="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C20="SI",C20="SÍ",C20=TRUE),"APROBADA",IF(OR(B20="SI",B20="SÍ",B20=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G20" s="9">
-        <f>IF(C20="SÍ","✅ Materia Aprobada",IF(B20="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C20="SI",C20="SÍ",C20=TRUE),"✅ Materia Aprobada",IF(OR(B20="SI",B20="SÍ",B20=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1271,15 +1271,15 @@
         </is>
       </c>
       <c r="E21" s="9">
-        <f>IF(B21="SÍ","CURSADA REGULAR",IF(AND(B5="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B21="SI",B21="SÍ",B21=TRUE),"CURSADA REGULAR",IF(AND(OR(B5="SI",B5="SÍ",B5=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F21" s="9">
-        <f>IF(C21="SÍ","APROBADA",IF(AND(B21="SÍ",AND(C5="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C21="SI",C21="SÍ",C21=TRUE),"APROBADA",IF(AND(OR(B21="SI",B21="SÍ",B21=TRUE),AND(OR(C5="SI",C5="SÍ",C5=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G21" s="9">
-        <f>IF(C21="SÍ","✅ Materia Aprobada",IF(B21="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C21="SI",C21="SÍ",C21=TRUE),"✅ Materia Aprobada",IF(OR(B21="SI",B21="SÍ",B21=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1305,15 +1305,15 @@
         </is>
       </c>
       <c r="E22" s="9">
-        <f>IF(B22="SÍ","CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B22="SI",B22="SÍ",B22=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
         <v/>
       </c>
       <c r="F22" s="9">
-        <f>IF(C22="SÍ","APROBADA",IF(B22="SÍ","¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C22="SI",C22="SÍ",C22=TRUE),"APROBADA",IF(OR(B22="SI",B22="SÍ",B22=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
         <v/>
       </c>
       <c r="G22" s="9">
-        <f>IF(C22="SÍ","✅ Materia Aprobada",IF(B22="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C22="SI",C22="SÍ",C22=TRUE),"✅ Materia Aprobada",IF(OR(B22="SI",B22="SÍ",B22=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1339,15 +1339,15 @@
         </is>
       </c>
       <c r="E23" s="9">
-        <f>IF(B23="SÍ","CURSADA REGULAR",IF(AND(B11="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B23="SI",B23="SÍ",B23=TRUE),"CURSADA REGULAR",IF(AND(OR(B11="SI",B11="SÍ",B11=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F23" s="9">
-        <f>IF(C23="SÍ","APROBADA",IF(AND(B23="SÍ",AND(C11="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C23="SI",C23="SÍ",C23=TRUE),"APROBADA",IF(AND(OR(B23="SI",B23="SÍ",B23=TRUE),AND(OR(C11="SI",C11="SÍ",C11=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G23" s="9">
-        <f>IF(C23="SÍ","✅ Materia Aprobada",IF(B23="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C23="SI",C23="SÍ",C23=TRUE),"✅ Materia Aprobada",IF(OR(B23="SI",B23="SÍ",B23=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1373,15 +1373,15 @@
         </is>
       </c>
       <c r="E24" s="9">
-        <f>IF(B24="SÍ","CURSADA REGULAR",IF(AND(B12="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B24="SI",B24="SÍ",B24=TRUE),"CURSADA REGULAR",IF(AND(OR(B12="SI",B12="SÍ",B12=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F24" s="9">
-        <f>IF(C24="SÍ","APROBADA",IF(AND(B24="SÍ",AND(C12="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C24="SI",C24="SÍ",C24=TRUE),"APROBADA",IF(AND(OR(B24="SI",B24="SÍ",B24=TRUE),AND(OR(C12="SI",C12="SÍ",C12=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G24" s="9">
-        <f>IF(C24="SÍ","✅ Materia Aprobada",IF(B24="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C24="SI",C24="SÍ",C24=TRUE),"✅ Materia Aprobada",IF(OR(B24="SI",B24="SÍ",B24=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1414,15 +1414,15 @@
         </is>
       </c>
       <c r="E26" s="9">
-        <f>IF(B26="SÍ","CURSADA REGULAR",IF(AND(B5="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B26="SI",B26="SÍ",B26=TRUE),"CURSADA REGULAR",IF(AND(OR(B5="SI",B5="SÍ",B5=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F26" s="9">
-        <f>IF(C26="SÍ","APROBADA",IF(AND(B26="SÍ",AND(C5="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C26="SI",C26="SÍ",C26=TRUE),"APROBADA",IF(AND(OR(B26="SI",B26="SÍ",B26=TRUE),AND(OR(C5="SI",C5="SÍ",C5=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G26" s="9">
-        <f>IF(C26="SÍ","✅ Materia Aprobada",IF(B26="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C26="SI",C26="SÍ",C26=TRUE),"✅ Materia Aprobada",IF(OR(B26="SI",B26="SÍ",B26=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1448,15 +1448,15 @@
         </is>
       </c>
       <c r="E27" s="9">
-        <f>IF(B27="SÍ","CURSADA REGULAR",IF(AND(B5="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B27="SI",B27="SÍ",B27=TRUE),"CURSADA REGULAR",IF(AND(OR(B5="SI",B5="SÍ",B5=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F27" s="9">
-        <f>IF(C27="SÍ","APROBADA",IF(AND(B27="SÍ",AND(C5="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C27="SI",C27="SÍ",C27=TRUE),"APROBADA",IF(AND(OR(B27="SI",B27="SÍ",B27=TRUE),AND(OR(C5="SI",C5="SÍ",C5=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G27" s="9">
-        <f>IF(C27="SÍ","✅ Materia Aprobada",IF(B27="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C27="SI",C27="SÍ",C27=TRUE),"✅ Materia Aprobada",IF(OR(B27="SI",B27="SÍ",B27=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1482,15 +1482,15 @@
         </is>
       </c>
       <c r="E28" s="9">
-        <f>IF(B28="SÍ","CURSADA REGULAR",IF(AND(B18="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B28="SI",B28="SÍ",B28=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F28" s="9">
-        <f>IF(C28="SÍ","APROBADA",IF(AND(B28="SÍ",AND(C18="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C28="SI",C28="SÍ",C28=TRUE),"APROBADA",IF(AND(OR(B28="SI",B28="SÍ",B28=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G28" s="9">
-        <f>IF(C28="SÍ","✅ Materia Aprobada",IF(B28="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C28="SI",C28="SÍ",C28=TRUE),"✅ Materia Aprobada",IF(OR(B28="SI",B28="SÍ",B28=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1516,15 +1516,15 @@
         </is>
       </c>
       <c r="E29" s="9">
-        <f>IF(B29="SÍ","CURSADA REGULAR",IF(AND(B18="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B29="SI",B29="SÍ",B29=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F29" s="9">
-        <f>IF(C29="SÍ","APROBADA",IF(AND(B29="SÍ",AND(C18="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C29="SI",C29="SÍ",C29=TRUE),"APROBADA",IF(AND(OR(B29="SI",B29="SÍ",B29=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G29" s="9">
-        <f>IF(C29="SÍ","✅ Materia Aprobada",IF(B29="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C29="SI",C29="SÍ",C29=TRUE),"✅ Materia Aprobada",IF(OR(B29="SI",B29="SÍ",B29=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1550,15 +1550,15 @@
         </is>
       </c>
       <c r="E30" s="9">
-        <f>IF(B30="SÍ","CURSADA REGULAR",IF(AND(B21="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B30="SI",B30="SÍ",B30=TRUE),"CURSADA REGULAR",IF(AND(OR(B21="SI",B21="SÍ",B21=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F30" s="9">
-        <f>IF(C30="SÍ","APROBADA",IF(AND(B30="SÍ",AND(C21="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C30="SI",C30="SÍ",C30=TRUE),"APROBADA",IF(AND(OR(B30="SI",B30="SÍ",B30=TRUE),AND(OR(C21="SI",C21="SÍ",C21=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G30" s="9">
-        <f>IF(C30="SÍ","✅ Materia Aprobada",IF(B30="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C30="SI",C30="SÍ",C30=TRUE),"✅ Materia Aprobada",IF(OR(B30="SI",B30="SÍ",B30=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1584,15 +1584,15 @@
         </is>
       </c>
       <c r="E31" s="9">
-        <f>IF(B31="SÍ","CURSADA REGULAR",IF(AND(B24="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B31="SI",B31="SÍ",B31=TRUE),"CURSADA REGULAR",IF(AND(OR(B24="SI",B24="SÍ",B24=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F31" s="9">
-        <f>IF(C31="SÍ","APROBADA",IF(AND(B31="SÍ",AND(C24="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C31="SI",C31="SÍ",C31=TRUE),"APROBADA",IF(AND(OR(B31="SI",B31="SÍ",B31=TRUE),AND(OR(C24="SI",C24="SÍ",C24=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G31" s="9">
-        <f>IF(C31="SÍ","✅ Materia Aprobada",IF(B31="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C31="SI",C31="SÍ",C31=TRUE),"✅ Materia Aprobada",IF(OR(B31="SI",B31="SÍ",B31=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1618,15 +1618,15 @@
         </is>
       </c>
       <c r="E32" s="9">
-        <f>IF(B32="SÍ","CURSADA REGULAR",IF(AND(B16="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B32="SI",B32="SÍ",B32=TRUE),"CURSADA REGULAR",IF(AND(OR(B16="SI",B16="SÍ",B16=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F32" s="9">
-        <f>IF(C32="SÍ","APROBADA",IF(AND(B32="SÍ",AND(C16="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C32="SI",C32="SÍ",C32=TRUE),"APROBADA",IF(AND(OR(B32="SI",B32="SÍ",B32=TRUE),AND(OR(C16="SI",C16="SÍ",C16=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G32" s="9">
-        <f>IF(C32="SÍ","✅ Materia Aprobada",IF(B32="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C32="SI",C32="SÍ",C32=TRUE),"✅ Materia Aprobada",IF(OR(B32="SI",B32="SÍ",B32=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1652,15 +1652,15 @@
         </is>
       </c>
       <c r="E33" s="9">
-        <f>IF(B33="SÍ","CURSADA REGULAR",IF(AND(B17="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B33="SI",B33="SÍ",B33=TRUE),"CURSADA REGULAR",IF(AND(OR(B17="SI",B17="SÍ",B17=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F33" s="9">
-        <f>IF(C33="SÍ","APROBADA",IF(AND(B33="SÍ",AND(C17="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C33="SI",C33="SÍ",C33=TRUE),"APROBADA",IF(AND(OR(B33="SI",B33="SÍ",B33=TRUE),AND(OR(C17="SI",C17="SÍ",C17=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G33" s="9">
-        <f>IF(C33="SÍ","✅ Materia Aprobada",IF(B33="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C33="SI",C33="SÍ",C33=TRUE),"✅ Materia Aprobada",IF(OR(B33="SI",B33="SÍ",B33=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1686,15 +1686,15 @@
         </is>
       </c>
       <c r="E34" s="9">
-        <f>IF(B34="SÍ","CURSADA REGULAR",IF(AND(B18="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B34="SI",B34="SÍ",B34=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F34" s="9">
-        <f>IF(C34="SÍ","APROBADA",IF(AND(B34="SÍ",AND(C18="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C34="SI",C34="SÍ",C34=TRUE),"APROBADA",IF(AND(OR(B34="SI",B34="SÍ",B34=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G34" s="9">
-        <f>IF(C34="SÍ","✅ Materia Aprobada",IF(B34="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C34="SI",C34="SÍ",C34=TRUE),"✅ Materia Aprobada",IF(OR(B34="SI",B34="SÍ",B34=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1720,15 +1720,15 @@
         </is>
       </c>
       <c r="E35" s="9">
-        <f>IF(B35="SÍ","CURSADA REGULAR",IF(AND(B18="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B35="SI",B35="SÍ",B35=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F35" s="9">
-        <f>IF(C35="SÍ","APROBADA",IF(AND(B35="SÍ",AND(C18="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C35="SI",C35="SÍ",C35=TRUE),"APROBADA",IF(AND(OR(B35="SI",B35="SÍ",B35=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G35" s="9">
-        <f>IF(C35="SÍ","✅ Materia Aprobada",IF(B35="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C35="SI",C35="SÍ",C35=TRUE),"✅ Materia Aprobada",IF(OR(B35="SI",B35="SÍ",B35=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1754,15 +1754,15 @@
         </is>
       </c>
       <c r="E36" s="9">
-        <f>IF(B36="SÍ","CURSADA REGULAR",IF(AND(B6="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B36="SI",B36="SÍ",B36=TRUE),"CURSADA REGULAR",IF(AND(OR(B6="SI",B6="SÍ",B6=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F36" s="9">
-        <f>IF(C36="SÍ","APROBADA",IF(AND(B36="SÍ",AND(C6="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C36="SI",C36="SÍ",C36=TRUE),"APROBADA",IF(AND(OR(B36="SI",B36="SÍ",B36=TRUE),AND(OR(C6="SI",C6="SÍ",C6=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G36" s="9">
-        <f>IF(C36="SÍ","✅ Materia Aprobada",IF(B36="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C36="SI",C36="SÍ",C36=TRUE),"✅ Materia Aprobada",IF(OR(B36="SI",B36="SÍ",B36=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1795,15 +1795,15 @@
         </is>
       </c>
       <c r="E38" s="9">
-        <f>IF(B38="SÍ","CURSADA REGULAR",IF(AND(B28="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B38="SI",B38="SÍ",B38=TRUE),"CURSADA REGULAR",IF(AND(OR(B28="SI",B28="SÍ",B28=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F38" s="9">
-        <f>IF(C38="SÍ","APROBADA",IF(AND(B38="SÍ",AND(C28="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C38="SI",C38="SÍ",C38=TRUE),"APROBADA",IF(AND(OR(B38="SI",B38="SÍ",B38=TRUE),AND(OR(C28="SI",C28="SÍ",C28=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G38" s="9">
-        <f>IF(C38="SÍ","✅ Materia Aprobada",IF(B38="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C38="SI",C38="SÍ",C38=TRUE),"✅ Materia Aprobada",IF(OR(B38="SI",B38="SÍ",B38=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1829,15 +1829,15 @@
         </is>
       </c>
       <c r="E39" s="9">
-        <f>IF(B39="SÍ","CURSADA REGULAR",IF(AND(B19="SÍ",B36="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B39="SI",B39="SÍ",B39=TRUE),"CURSADA REGULAR",IF(AND(OR(B19="SI",B19="SÍ",B19=TRUE),OR(B36="SI",B36="SÍ",B36=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F39" s="9">
-        <f>IF(C39="SÍ","APROBADA",IF(AND(B39="SÍ",AND(C19="SÍ",C36="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C39="SI",C39="SÍ",C39=TRUE),"APROBADA",IF(AND(OR(B39="SI",B39="SÍ",B39=TRUE),AND(OR(C19="SI",C19="SÍ",C19=TRUE),OR(C36="SI",C36="SÍ",C36=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G39" s="9">
-        <f>IF(C39="SÍ","✅ Materia Aprobada",IF(B39="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C39="SI",C39="SÍ",C39=TRUE),"✅ Materia Aprobada",IF(OR(B39="SI",B39="SÍ",B39=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1863,15 +1863,15 @@
         </is>
       </c>
       <c r="E40" s="9">
-        <f>IF(B40="SÍ","CURSADA REGULAR",IF(AND(B27="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B40="SI",B40="SÍ",B40=TRUE),"CURSADA REGULAR",IF(AND(OR(B27="SI",B27="SÍ",B27=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F40" s="9">
-        <f>IF(C40="SÍ","APROBADA",IF(AND(B40="SÍ",AND(C27="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C40="SI",C40="SÍ",C40=TRUE),"APROBADA",IF(AND(OR(B40="SI",B40="SÍ",B40=TRUE),AND(OR(C27="SI",C27="SÍ",C27=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G40" s="9">
-        <f>IF(C40="SÍ","✅ Materia Aprobada",IF(B40="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C40="SI",C40="SÍ",C40=TRUE),"✅ Materia Aprobada",IF(OR(B40="SI",B40="SÍ",B40=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1897,15 +1897,15 @@
         </is>
       </c>
       <c r="E41" s="9">
-        <f>IF(B41="SÍ","CURSADA REGULAR",IF(AND(B18="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B41="SI",B41="SÍ",B41=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F41" s="9">
-        <f>IF(C41="SÍ","APROBADA",IF(AND(B41="SÍ",AND(C18="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C41="SI",C41="SÍ",C41=TRUE),"APROBADA",IF(AND(OR(B41="SI",B41="SÍ",B41=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G41" s="9">
-        <f>IF(C41="SÍ","✅ Materia Aprobada",IF(B41="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C41="SI",C41="SÍ",C41=TRUE),"✅ Materia Aprobada",IF(OR(B41="SI",B41="SÍ",B41=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1931,15 +1931,15 @@
         </is>
       </c>
       <c r="E42" s="9">
-        <f>IF(B42="SÍ","CURSADA REGULAR",IF(AND(B20="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B42="SI",B42="SÍ",B42=TRUE),"CURSADA REGULAR",IF(AND(OR(B20="SI",B20="SÍ",B20=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F42" s="9">
-        <f>IF(C42="SÍ","APROBADA",IF(AND(B42="SÍ",AND(C20="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C42="SI",C42="SÍ",C42=TRUE),"APROBADA",IF(AND(OR(B42="SI",B42="SÍ",B42=TRUE),AND(OR(C20="SI",C20="SÍ",C20=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G42" s="9">
-        <f>IF(C42="SÍ","✅ Materia Aprobada",IF(B42="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C42="SI",C42="SÍ",C42=TRUE),"✅ Materia Aprobada",IF(OR(B42="SI",B42="SÍ",B42=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -1965,15 +1965,15 @@
         </is>
       </c>
       <c r="E43" s="9">
-        <f>IF(B43="SÍ","CURSADA REGULAR",IF(AND(B32="SÍ",B31="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B43="SI",B43="SÍ",B43=TRUE),"CURSADA REGULAR",IF(AND(OR(B32="SI",B32="SÍ",B32=TRUE),OR(B31="SI",B31="SÍ",B31=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F43" s="9">
-        <f>IF(C43="SÍ","APROBADA",IF(AND(B43="SÍ",AND(C32="SÍ",C31="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C43="SI",C43="SÍ",C43=TRUE),"APROBADA",IF(AND(OR(B43="SI",B43="SÍ",B43=TRUE),AND(OR(C32="SI",C32="SÍ",C32=TRUE),OR(C31="SI",C31="SÍ",C31=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G43" s="9">
-        <f>IF(C43="SÍ","✅ Materia Aprobada",IF(B43="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C43="SI",C43="SÍ",C43=TRUE),"✅ Materia Aprobada",IF(OR(B43="SI",B43="SÍ",B43=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2006,15 +2006,15 @@
         </is>
       </c>
       <c r="E45" s="9">
-        <f>IF(B45="SÍ","CURSADA REGULAR",IF(AND(B38="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B45="SI",B45="SÍ",B45=TRUE),"CURSADA REGULAR",IF(AND(OR(B38="SI",B38="SÍ",B38=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F45" s="9">
-        <f>IF(C45="SÍ","APROBADA",IF(AND(B45="SÍ",AND(C38="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C45="SI",C45="SÍ",C45=TRUE),"APROBADA",IF(AND(OR(B45="SI",B45="SÍ",B45=TRUE),AND(OR(C38="SI",C38="SÍ",C38=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G45" s="9">
-        <f>IF(C45="SÍ","✅ Materia Aprobada",IF(B45="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C45="SI",C45="SÍ",C45=TRUE),"✅ Materia Aprobada",IF(OR(B45="SI",B45="SÍ",B45=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2040,15 +2040,15 @@
         </is>
       </c>
       <c r="E46" s="9">
-        <f>IF(B46="SÍ","CURSADA REGULAR",IF(AND(B39="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B46="SI",B46="SÍ",B46=TRUE),"CURSADA REGULAR",IF(AND(OR(B39="SI",B39="SÍ",B39=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F46" s="9">
-        <f>IF(C46="SÍ","APROBADA",IF(AND(B46="SÍ",AND(C39="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C46="SI",C46="SÍ",C46=TRUE),"APROBADA",IF(AND(OR(B46="SI",B46="SÍ",B46=TRUE),AND(OR(C39="SI",C39="SÍ",C39=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G46" s="9">
-        <f>IF(C46="SÍ","✅ Materia Aprobada",IF(B46="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C46="SI",C46="SÍ",C46=TRUE),"✅ Materia Aprobada",IF(OR(B46="SI",B46="SÍ",B46=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2074,15 +2074,15 @@
         </is>
       </c>
       <c r="E47" s="9">
-        <f>IF(B47="SÍ","CURSADA REGULAR",IF(AND(B28="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B47="SI",B47="SÍ",B47=TRUE),"CURSADA REGULAR",IF(AND(OR(B28="SI",B28="SÍ",B28=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F47" s="9">
-        <f>IF(C47="SÍ","APROBADA",IF(AND(B47="SÍ",AND(C28="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C47="SI",C47="SÍ",C47=TRUE),"APROBADA",IF(AND(OR(B47="SI",B47="SÍ",B47=TRUE),AND(OR(C28="SI",C28="SÍ",C28=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G47" s="9">
-        <f>IF(C47="SÍ","✅ Materia Aprobada",IF(B47="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C47="SI",C47="SÍ",C47=TRUE),"✅ Materia Aprobada",IF(OR(B47="SI",B47="SÍ",B47=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2108,15 +2108,15 @@
         </is>
       </c>
       <c r="E48" s="9">
-        <f>IF(B48="SÍ","CURSADA REGULAR",IF(AND(B38="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B48="SI",B48="SÍ",B48=TRUE),"CURSADA REGULAR",IF(AND(OR(B38="SI",B38="SÍ",B38=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F48" s="9">
-        <f>IF(C48="SÍ","APROBADA",IF(AND(B48="SÍ",AND(C38="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C48="SI",C48="SÍ",C48=TRUE),"APROBADA",IF(AND(OR(B48="SI",B48="SÍ",B48=TRUE),AND(OR(C38="SI",C38="SÍ",C38=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G48" s="9">
-        <f>IF(C48="SÍ","✅ Materia Aprobada",IF(B48="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C48="SI",C48="SÍ",C48=TRUE),"✅ Materia Aprobada",IF(OR(B48="SI",B48="SÍ",B48=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2142,15 +2142,15 @@
         </is>
       </c>
       <c r="E49" s="9">
-        <f>IF(B49="SÍ","CURSADA REGULAR",IF(AND(B30="SÍ",B35="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B49="SI",B49="SÍ",B49=TRUE),"CURSADA REGULAR",IF(AND(OR(B30="SI",B30="SÍ",B30=TRUE),OR(B35="SI",B35="SÍ",B35=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F49" s="9">
-        <f>IF(C49="SÍ","APROBADA",IF(AND(B49="SÍ",AND(C30="SÍ",C35="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C49="SI",C49="SÍ",C49=TRUE),"APROBADA",IF(AND(OR(B49="SI",B49="SÍ",B49=TRUE),AND(OR(C30="SI",C30="SÍ",C30=TRUE),OR(C35="SI",C35="SÍ",C35=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G49" s="9">
-        <f>IF(C49="SÍ","✅ Materia Aprobada",IF(B49="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C49="SI",C49="SÍ",C49=TRUE),"✅ Materia Aprobada",IF(OR(B49="SI",B49="SÍ",B49=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2176,15 +2176,15 @@
         </is>
       </c>
       <c r="E50" s="9">
-        <f>IF(B50="SÍ","CURSADA REGULAR",IF(AND(B43="SÍ"),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B50="SI",B50="SÍ",B50=TRUE),"CURSADA REGULAR",IF(AND(OR(B43="SI",B43="SÍ",B43=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
         <v/>
       </c>
       <c r="F50" s="9">
-        <f>IF(C50="SÍ","APROBADA",IF(AND(B50="SÍ",AND(C43="SÍ")),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C50="SI",C50="SÍ",C50=TRUE),"APROBADA",IF(AND(OR(B50="SI",B50="SÍ",B50=TRUE),AND(OR(C43="SI",C43="SÍ",C43=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
         <v/>
       </c>
       <c r="G50" s="9">
-        <f>IF(C50="SÍ","✅ Materia Aprobada",IF(B50="SÍ","⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C50="SI",C50="SÍ",C50=TRUE),"✅ Materia Aprobada",IF(OR(B50="SI",B50="SÍ",B50=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2205,6 +2205,11 @@
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="A37:G37"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B4:C50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SI,NO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(mapa): menu desplegable nativo para SI/NO e instrucciones de Supabase
</commit_message>
<xml_diff>
--- a/data/mapas/Mapa_de_Carrera_Filosofia.xlsx
+++ b/data/mapas/Mapa_de_Carrera_Filosofia.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa de Carrera" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opciones" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -576,8 +577,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -608,12 +609,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>¿Cursada Regular? (SI / NO)</t>
+          <t>¿Cursada Regular? (Elegir SI/NO)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>¿Final Aprobado? (SI / NO)</t>
+          <t>¿Final Aprobado? (Elegir SI/NO)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -945,7 +946,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="26" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Trabajo de Campo 1</t>
@@ -980,11 +981,11 @@
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
-          <t>1. Seleccioná 'SI' o 'SÍ' en la columna B cuando tengas la cursada regular aprobada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
+          <t>1. Hacé clic en la celda y elegí 'SI' o 'NO' desde el menú desplegable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Educación Sexual Integral (ESI)</t>
@@ -1019,11 +1020,11 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>2. Seleccioná 'SI' o 'SÍ' en la columna C cuando hayas aprobado el examen final.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
+          <t>2. Columna B: Marcá 'SI' si tenés la cursada regular aprobada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Lengua Extranjera</t>
@@ -1058,11 +1059,11 @@
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
-          <t>3. Las columnas E y F te dirán automáticamente si estás en condiciones de cursar o rendir cada materia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
+          <t>3. Columna C: Marcá 'SI' si aprobaste el final o promocionaste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>📌 SEGUNDO AÑO</t>
@@ -1070,11 +1071,11 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>4. El panel de la derecha calcula tus porcentajes en tiempo real.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
+          <t>4. Las columnas E y F te informan automáticamente qué podés cursar o rendir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Didáctica General</t>
@@ -1109,11 +1110,11 @@
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>5. ¡Guardá una copia en tu Google Drive personal para no perder tus avances!</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
+          <t>5. El panel lateral calcula tu avance y porcentaje de carrera en tiempo real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Historia de la Educación Argentina</t>
@@ -1146,6 +1147,11 @@
         <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"✅ Materia Aprobada",IF(OR(B17="SI",B17="SÍ",B17=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>6. Guardá una copia en tu Google Drive personal para conservar tus progresos.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
@@ -2189,7 +2195,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="I14:J14"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="I12:J12"/>
@@ -2203,13 +2209,42 @@
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="A25:G25"/>
+    <mergeCell ref="I17:J17"/>
     <mergeCell ref="A37:G37"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B4:C50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SI,NO"</formula1>
+    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B16 B17 B18 B19 B20 B21 B22 B23 B24 B26 B27 B28 B29 B30 B31 B32 B33 B34 B35 B36 B38 B39 B40 B41 B42 B43 B45 B46 B47 B48 B49 B50 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C16 C17 C18 C19 C20 C21 C22 C23 C24 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C38 C39 C40 C41 C42 C43 C45 C46 C47 C48 C49 C50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Opción no válida" error="Elegí una opción de la lista" promptTitle="Estado de Materia" prompt="Elegí SI o NO" type="list">
+      <formula1>=Opciones!$A$1:$A$2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(mapa): menu desplegable nativo visible con sqref B5:C50 y eliminacion de showDropDown=0
</commit_message>
<xml_diff>
--- a/data/mapas/Mapa_de_Carrera_Filosofia.xlsx
+++ b/data/mapas/Mapa_de_Carrera_Filosofia.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa de Carrera" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opciones" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2213,38 +2212,10 @@
     <mergeCell ref="A37:G37"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B16 B17 B18 B19 B20 B21 B22 B23 B24 B26 B27 B28 B29 B30 B31 B32 B33 B34 B35 B36 B38 B39 B40 B41 B42 B43 B45 B46 B47 B48 B49 B50 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C16 C17 C18 C19 C20 C21 C22 C23 C24 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C38 C39 C40 C41 C42 C43 C45 C46 C47 C48 C49 C50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Opción no válida" error="Elegí una opción de la lista" promptTitle="Estado de Materia" prompt="Elegí SI o NO" type="list">
-      <formula1>=Opciones!$A$1:$A$2</formula1>
+    <dataValidation sqref="B5:C50" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: comodato computadoras, newsletter de avisos, buzon admin, terminos legales y mapas de carrera
</commit_message>
<xml_diff>
--- a/data/mapas/Mapa_de_Carrera_Filosofia.xlsx
+++ b/data/mapas/Mapa_de_Carrera_Filosofia.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,7 +31,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -62,13 +62,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
       <color rgb="0064748B"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000F172A"/>
       <sz val="9"/>
     </font>
     <font>
@@ -154,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -174,7 +168,7 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,15 +178,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -200,12 +194,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,16 +560,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
@@ -589,14 +577,14 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MAPA DE CARRERA PERSONAL | ALTILLO JVG</t>
+          <t>MAPA DE CARRERA | PROFESORADO DE FILOSOFÍA</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Desarrollado por La Caravana + Estudiantes Independientes (Lista 90) - Joaquín V. González</t>
+          <t>La Caravana + Estudiantes Independientes | Altillo JVG - ISP Joaquín V. González</t>
         </is>
       </c>
     </row>
@@ -608,32 +596,32 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>¿Cursada Regular? (Elegir SI/NO)</t>
+          <t>¿Cursada Regular? (SI/NO)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>¿Final Aprobado? (Elegir SI/NO)</t>
+          <t>¿Final Aprobado? (SI/NO)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Correlativas para Cursar</t>
+          <t>Régimen / Año</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>¿Podés Cursar?</t>
+          <t>¿Cursada?</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>¿Podés Rendir Final?</t>
+          <t>¿Final?</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Estado Trayectoria</t>
+          <t>Estado de Avance</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -645,7 +633,7 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>📌 PRIMER AÑO</t>
+          <t>📌 1° AÑO</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -654,13 +642,13 @@
         </is>
       </c>
       <c r="J4" s="7" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Lógica 1 y Teoría de la Argumentación</t>
+          <t>INTRODUCCION A LA FILOSOFIA</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
@@ -675,19 +663,19 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E5" s="9">
-        <f>IF(OR(B5="SI",B5="SÍ",B5=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B5="SI",B5="SÍ",B5=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F5" s="9">
-        <f>IF(OR(C5="SI",C5="SÍ",C5=TRUE),"APROBADA",IF(OR(B5="SI",B5="SÍ",B5=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C5="SI",C5="SÍ",C5=TRUE),"APROBADA",IF(OR(B5="SI",B5="SÍ",B5=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G5" s="9">
-        <f>IF(OR(C5="SI",C5="SÍ",C5=TRUE),"✅ Materia Aprobada",IF(OR(B5="SI",B5="SÍ",B5=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C5="SI",C5="SÍ",C5=TRUE),"✅ Aprobada",IF(OR(B5="SI",B5="SÍ",B5=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -696,14 +684,14 @@
         </is>
       </c>
       <c r="J5" s="7">
-        <f>COUNTIF(B4:B50, "S*") + COUNTIF(B4:B50, TRUE)</f>
+        <f>COUNTIF(B4:B54, "S*") + COUNTIF(B4:B54, TRUE)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Introducción a la Filosofía</t>
+          <t>LECTURA, ESCRITURA Y ORALIDAD I</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -718,19 +706,19 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E6" s="9">
-        <f>IF(OR(B6="SI",B6="SÍ",B6=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B6="SI",B6="SÍ",B6=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>IF(OR(C6="SI",C6="SÍ",C6=TRUE),"APROBADA",IF(OR(B6="SI",B6="SÍ",B6=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C6="SI",C6="SÍ",C6=TRUE),"APROBADA",IF(OR(B6="SI",B6="SÍ",B6=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G6" s="9">
-        <f>IF(OR(C6="SI",C6="SÍ",C6=TRUE),"✅ Materia Aprobada",IF(OR(B6="SI",B6="SÍ",B6=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C6="SI",C6="SÍ",C6=TRUE),"✅ Aprobada",IF(OR(B6="SI",B6="SÍ",B6=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -739,14 +727,14 @@
         </is>
       </c>
       <c r="J6" s="7">
-        <f>COUNTIF(C4:C50, "S*") + COUNTIF(C4:C50, TRUE)</f>
+        <f>COUNTIF(C4:C54, "S*") + COUNTIF(C4:C54, TRUE)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Psicología Educacional</t>
+          <t>LOGICA I Y TEORIA DE LA ARGUMENTACION</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -761,19 +749,19 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E7" s="9">
-        <f>IF(OR(B7="SI",B7="SÍ",B7=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B7="SI",B7="SÍ",B7=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>IF(OR(C7="SI",C7="SÍ",C7=TRUE),"APROBADA",IF(OR(B7="SI",B7="SÍ",B7=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C7="SI",C7="SÍ",C7=TRUE),"APROBADA",IF(OR(B7="SI",B7="SÍ",B7=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>IF(OR(C7="SI",C7="SÍ",C7=TRUE),"✅ Materia Aprobada",IF(OR(B7="SI",B7="SÍ",B7=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C7="SI",C7="SÍ",C7=TRUE),"✅ Aprobada",IF(OR(B7="SI",B7="SÍ",B7=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -789,7 +777,7 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Psicología del Desarrollo</t>
+          <t>PEDAGOGIA</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -804,19 +792,19 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E8" s="9">
-        <f>IF(OR(B8="SI",B8="SÍ",B8=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B8="SI",B8="SÍ",B8=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>IF(OR(C8="SI",C8="SÍ",C8=TRUE),"APROBADA",IF(OR(B8="SI",B8="SÍ",B8=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C8="SI",C8="SÍ",C8=TRUE),"APROBADA",IF(OR(B8="SI",B8="SÍ",B8=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>IF(OR(C8="SI",C8="SÍ",C8=TRUE),"✅ Materia Aprobada",IF(OR(B8="SI",B8="SÍ",B8=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C8="SI",C8="SÍ",C8=TRUE),"✅ Aprobada",IF(OR(B8="SI",B8="SÍ",B8=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -825,14 +813,14 @@
         </is>
       </c>
       <c r="J8" s="13">
-        <f>J5/42</f>
+        <f>J5/45</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Sociología</t>
+          <t>PSICOLOGIA EDUCACIONAL (1° Cuat.)</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -847,19 +835,19 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E9" s="9">
-        <f>IF(OR(B9="SI",B9="SÍ",B9=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B9="SI",B9="SÍ",B9=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>IF(OR(C9="SI",C9="SÍ",C9=TRUE),"APROBADA",IF(OR(B9="SI",B9="SÍ",B9=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C9="SI",C9="SÍ",C9=TRUE),"APROBADA",IF(OR(B9="SI",B9="SÍ",B9=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>IF(OR(C9="SI",C9="SÍ",C9=TRUE),"✅ Materia Aprobada",IF(OR(B9="SI",B9="SÍ",B9=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C9="SI",C9="SÍ",C9=TRUE),"✅ Aprobada",IF(OR(B9="SI",B9="SÍ",B9=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -868,14 +856,14 @@
         </is>
       </c>
       <c r="J9" s="13">
-        <f>J6/42</f>
+        <f>J6/45</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Pedagogía</t>
+          <t>SOCIOLOGIA</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -890,26 +878,26 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E10" s="9">
-        <f>IF(OR(B10="SI",B10="SÍ",B10=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B10="SI",B10="SÍ",B10=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>IF(OR(C10="SI",C10="SÍ",C10=TRUE),"APROBADA",IF(OR(B10="SI",B10="SÍ",B10=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C10="SI",C10="SÍ",C10=TRUE),"APROBADA",IF(OR(B10="SI",B10="SÍ",B10=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G10" s="9">
-        <f>IF(OR(C10="SI",C10="SÍ",C10=TRUE),"✅ Materia Aprobada",IF(OR(B10="SI",B10="SÍ",B10=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C10="SI",C10="SÍ",C10=TRUE),"✅ Aprobada",IF(OR(B10="SI",B10="SÍ",B10=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>LEO 1 (Lectura y Escritura Académica)</t>
+          <t>TRABAJO DE CAMPO I</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -924,19 +912,19 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E11" s="9">
-        <f>IF(OR(B11="SI",B11="SÍ",B11=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B11="SI",B11="SÍ",B11=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F11" s="9">
-        <f>IF(OR(C11="SI",C11="SÍ",C11=TRUE),"APROBADA",IF(OR(B11="SI",B11="SÍ",B11=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C11="SI",C11="SÍ",C11=TRUE),"APROBADA",IF(OR(B11="SI",B11="SÍ",B11=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G11" s="9">
-        <f>IF(OR(C11="SI",C11="SÍ",C11=TRUE),"✅ Materia Aprobada",IF(OR(B11="SI",B11="SÍ",B11=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C11="SI",C11="SÍ",C11=TRUE),"✅ Aprobada",IF(OR(B11="SI",B11="SÍ",B11=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I11" s="14" t="inlineStr">
@@ -946,37 +934,10 @@
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Trabajo de Campo 1</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Sin correlativas previas</t>
-        </is>
-      </c>
-      <c r="E12" s="9">
-        <f>IF(OR(B12="SI",B12="SÍ",B12=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
-        <v/>
-      </c>
-      <c r="F12" s="9">
-        <f>IF(OR(C12="SI",C12="SÍ",C12=TRUE),"APROBADA",IF(OR(B12="SI",B12="SÍ",B12=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
-        <v/>
-      </c>
-      <c r="G12" s="9">
-        <f>IF(OR(C12="SI",C12="SÍ",C12=TRUE),"✅ Materia Aprobada",IF(OR(B12="SI",B12="SÍ",B12=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>📌 2° AÑO</t>
+        </is>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
@@ -987,7 +948,7 @@
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Educación Sexual Integral (ESI)</t>
+          <t>DIDACTICA GENERAL</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
@@ -1002,19 +963,19 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E13" s="9">
-        <f>IF(OR(B13="SI",B13="SÍ",B13=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B13="SI",B13="SÍ",B13=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>IF(OR(C13="SI",C13="SÍ",C13=TRUE),"APROBADA",IF(OR(B13="SI",B13="SÍ",B13=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C13="SI",C13="SÍ",C13=TRUE),"APROBADA",IF(OR(B13="SI",B13="SÍ",B13=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G13" s="9">
-        <f>IF(OR(C13="SI",C13="SÍ",C13=TRUE),"✅ Materia Aprobada",IF(OR(B13="SI",B13="SÍ",B13=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C13="SI",C13="SÍ",C13=TRUE),"✅ Aprobada",IF(OR(B13="SI",B13="SÍ",B13=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I13" s="15" t="inlineStr">
@@ -1026,7 +987,7 @@
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Lengua Extranjera</t>
+          <t>FILOSOFIA ARGENTINA Y LATINOAMERICANA</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -1041,19 +1002,19 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E14" s="9">
-        <f>IF(OR(B14="SI",B14="SÍ",B14=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B14="SI",B14="SÍ",B14=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>IF(OR(C14="SI",C14="SÍ",C14=TRUE),"APROBADA",IF(OR(B14="SI",B14="SÍ",B14=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C14="SI",C14="SÍ",C14=TRUE),"APROBADA",IF(OR(B14="SI",B14="SÍ",B14=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>IF(OR(C14="SI",C14="SÍ",C14=TRUE),"✅ Materia Aprobada",IF(OR(B14="SI",B14="SÍ",B14=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C14="SI",C14="SÍ",C14=TRUE),"✅ Aprobada",IF(OR(B14="SI",B14="SÍ",B14=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I14" s="15" t="inlineStr">
@@ -1063,21 +1024,48 @@
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>📌 SEGUNDO AÑO</t>
-        </is>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>HISTORIA DE LA EDUCACION ARGENTINA</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>2° Año</t>
+        </is>
+      </c>
+      <c r="E15" s="9">
+        <f>IF(OR(B15="SI",B15="SÍ",B15=TRUE),"REGULAR","PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F15" s="9">
+        <f>IF(OR(C15="SI",C15="SÍ",C15=TRUE),"APROBADA",IF(OR(B15="SI",B15="SÍ",B15=TRUE),"RINDE FINAL","ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G15" s="9">
+        <f>IF(OR(C15="SI",C15="SÍ",C15=TRUE),"✅ Aprobada",IF(OR(B15="SI",B15="SÍ",B15=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>4. Las columnas E y F te informan automáticamente qué podés cursar o rendir.</t>
+          <t>4. Las columnas E, F y G se actualizan automáticamente en tiempo real.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Didáctica General</t>
+          <t>HISTORIA DE LA FILOSOFIA ANTIGUA</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -1090,33 +1078,33 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>Pedagogía</t>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E16" s="9">
-        <f>IF(OR(B16="SI",B16="SÍ",B16=TRUE),"CURSADA REGULAR",IF(AND(OR(B10="SI",B10="SÍ",B10=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B16="SI",B16="SÍ",B16=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>IF(OR(C16="SI",C16="SÍ",C16=TRUE),"APROBADA",IF(AND(OR(B16="SI",B16="SÍ",B16=TRUE),AND(OR(C10="SI",C10="SÍ",C10=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C16="SI",C16="SÍ",C16=TRUE),"APROBADA",IF(OR(B16="SI",B16="SÍ",B16=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G16" s="9">
-        <f>IF(OR(C16="SI",C16="SÍ",C16=TRUE),"✅ Materia Aprobada",IF(OR(B16="SI",B16="SÍ",B16=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C16="SI",C16="SÍ",C16=TRUE),"✅ Aprobada",IF(OR(B16="SI",B16="SÍ",B16=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>5. El panel lateral calcula tu avance y porcentaje de carrera en tiempo real.</t>
+          <t>5. El panel lateral calcula tu avance y porcentaje de carrera en vivo.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Historia de la Educación Argentina</t>
+          <t>HISTORIA DEL ARTE</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -1129,33 +1117,33 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
-        <is>
-          <t>Pedagogía, Sociología</t>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E17" s="9">
-        <f>IF(OR(B17="SI",B17="SÍ",B17=TRUE),"CURSADA REGULAR",IF(AND(OR(B10="SI",B10="SÍ",B10=TRUE),OR(B9="SI",B9="SÍ",B9=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B17="SI",B17="SÍ",B17=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F17" s="9">
-        <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"APROBADA",IF(AND(OR(B17="SI",B17="SÍ",B17=TRUE),AND(OR(C10="SI",C10="SÍ",C10=TRUE),OR(C9="SI",C9="SÍ",C9=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"APROBADA",IF(OR(B17="SI",B17="SÍ",B17=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G17" s="9">
-        <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"✅ Materia Aprobada",IF(OR(B17="SI",B17="SÍ",B17=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"✅ Aprobada",IF(OR(B17="SI",B17="SÍ",B17=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>6. Guardá una copia en tu Google Drive personal para conservar tus progresos.</t>
+          <t>6. Podés subir el archivo a tu Google Drive personal para editarlo online.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Historia de la Filosofía Antigua</t>
+          <t>LECTURA, ESCRITA Y ORALIDAD II</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -1168,28 +1156,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>Introducción a la Filosofía</t>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E18" s="9">
-        <f>IF(OR(B18="SI",B18="SÍ",B18=TRUE),"CURSADA REGULAR",IF(AND(OR(B6="SI",B6="SÍ",B6=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B18="SI",B18="SÍ",B18=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>IF(OR(C18="SI",C18="SÍ",C18=TRUE),"APROBADA",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE),AND(OR(C6="SI",C6="SÍ",C6=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C18="SI",C18="SÍ",C18=TRUE),"APROBADA",IF(OR(B18="SI",B18="SÍ",B18=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>IF(OR(C18="SI",C18="SÍ",C18=TRUE),"✅ Materia Aprobada",IF(OR(B18="SI",B18="SÍ",B18=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C18="SI",C18="SÍ",C18=TRUE),"✅ Aprobada",IF(OR(B18="SI",B18="SÍ",B18=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Filosofía Argentina y Latinoamericana</t>
+          <t>METODOLOGIA DE LA INVESTIGACION</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -1202,28 +1190,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
-        <is>
-          <t>Introducción a la Filosofía</t>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E19" s="9">
-        <f>IF(OR(B19="SI",B19="SÍ",B19=TRUE),"CURSADA REGULAR",IF(AND(OR(B6="SI",B6="SÍ",B6=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B19="SI",B19="SÍ",B19=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F19" s="9">
-        <f>IF(OR(C19="SI",C19="SÍ",C19=TRUE),"APROBADA",IF(AND(OR(B19="SI",B19="SÍ",B19=TRUE),AND(OR(C6="SI",C6="SÍ",C6=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C19="SI",C19="SÍ",C19=TRUE),"APROBADA",IF(OR(B19="SI",B19="SÍ",B19=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G19" s="9">
-        <f>IF(OR(C19="SI",C19="SÍ",C19=TRUE),"✅ Materia Aprobada",IF(OR(B19="SI",B19="SÍ",B19=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C19="SI",C19="SÍ",C19=TRUE),"✅ Aprobada",IF(OR(B19="SI",B19="SÍ",B19=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Historia del Arte</t>
+          <t>NUEVAS TECNOLOGIAS (1° CUATR.)</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -1238,26 +1226,26 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Sin correlativas previas</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E20" s="9">
-        <f>IF(OR(B20="SI",B20="SÍ",B20=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
+        <f>IF(OR(B20="SI",B20="SÍ",B20=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>IF(OR(C20="SI",C20="SÍ",C20=TRUE),"APROBADA",IF(OR(B20="SI",B20="SÍ",B20=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
+        <f>IF(OR(C20="SI",C20="SÍ",C20=TRUE),"APROBADA",IF(OR(B20="SI",B20="SÍ",B20=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G20" s="9">
-        <f>IF(OR(C20="SI",C20="SÍ",C20=TRUE),"✅ Materia Aprobada",IF(OR(B20="SI",B20="SÍ",B20=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C20="SI",C20="SÍ",C20=TRUE),"✅ Aprobada",IF(OR(B20="SI",B20="SÍ",B20=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Metodología de la Investigación</t>
+          <t>TRABAJO DE CAMPO II</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -1270,62 +1258,35 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
-        <is>
-          <t>Lógica 1 y Teoría de la Argumentación</t>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E21" s="9">
-        <f>IF(OR(B21="SI",B21="SÍ",B21=TRUE),"CURSADA REGULAR",IF(AND(OR(B5="SI",B5="SÍ",B5=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B21="SI",B21="SÍ",B21=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F21" s="9">
-        <f>IF(OR(C21="SI",C21="SÍ",C21=TRUE),"APROBADA",IF(AND(OR(B21="SI",B21="SÍ",B21=TRUE),AND(OR(C5="SI",C5="SÍ",C5=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C21="SI",C21="SÍ",C21=TRUE),"APROBADA",IF(OR(B21="SI",B21="SÍ",B21=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G21" s="9">
-        <f>IF(OR(C21="SI",C21="SÍ",C21=TRUE),"✅ Materia Aprobada",IF(OR(B21="SI",B21="SÍ",B21=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Nuevas Tecnologías</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Sin correlativas previas</t>
-        </is>
-      </c>
-      <c r="E22" s="9">
-        <f>IF(OR(B22="SI",B22="SÍ",B22=TRUE),"CURSADA REGULAR","¡HABILITADA!")</f>
-        <v/>
-      </c>
-      <c r="F22" s="9">
-        <f>IF(OR(C22="SI",C22="SÍ",C22=TRUE),"APROBADA",IF(OR(B22="SI",B22="SÍ",B22=TRUE),"¡LISTO P/ FINAL!","Falta cursada"))</f>
-        <v/>
-      </c>
-      <c r="G22" s="9">
-        <f>IF(OR(C22="SI",C22="SÍ",C22=TRUE),"✅ Materia Aprobada",IF(OR(B22="SI",B22="SÍ",B22=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
+        <f>IF(OR(C21="SI",C21="SÍ",C21=TRUE),"✅ Aprobada",IF(OR(B21="SI",B21="SÍ",B21=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>📌 3° AÑO</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>LEO 2</t>
+          <t>ETICA</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -1338,28 +1299,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
-        <is>
-          <t>LEO 1 (Lectura y Escritura Académica)</t>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E23" s="9">
-        <f>IF(OR(B23="SI",B23="SÍ",B23=TRUE),"CURSADA REGULAR",IF(AND(OR(B11="SI",B11="SÍ",B11=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B23="SI",B23="SÍ",B23=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F23" s="9">
-        <f>IF(OR(C23="SI",C23="SÍ",C23=TRUE),"APROBADA",IF(AND(OR(B23="SI",B23="SÍ",B23=TRUE),AND(OR(C11="SI",C11="SÍ",C11=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C23="SI",C23="SÍ",C23=TRUE),"APROBADA",IF(OR(B23="SI",B23="SÍ",B23=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G23" s="9">
-        <f>IF(OR(C23="SI",C23="SÍ",C23=TRUE),"✅ Materia Aprobada",IF(OR(B23="SI",B23="SÍ",B23=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C23="SI",C23="SÍ",C23=TRUE),"✅ Aprobada",IF(OR(B23="SI",B23="SÍ",B23=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Trabajo de Campo 2</t>
+          <t>HISTORIA DE LA CIENCIA "A"</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -1372,35 +1333,62 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>Trabajo de Campo 1</t>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E24" s="9">
-        <f>IF(OR(B24="SI",B24="SÍ",B24=TRUE),"CURSADA REGULAR",IF(AND(OR(B12="SI",B12="SÍ",B12=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B24="SI",B24="SÍ",B24=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F24" s="9">
-        <f>IF(OR(C24="SI",C24="SÍ",C24=TRUE),"APROBADA",IF(AND(OR(B24="SI",B24="SÍ",B24=TRUE),AND(OR(C12="SI",C12="SÍ",C12=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C24="SI",C24="SÍ",C24=TRUE),"APROBADA",IF(OR(B24="SI",B24="SÍ",B24=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G24" s="9">
-        <f>IF(OR(C24="SI",C24="SÍ",C24=TRUE),"✅ Materia Aprobada",IF(OR(B24="SI",B24="SÍ",B24=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>📌 TERCER AÑO</t>
-        </is>
+        <f>IF(OR(C24="SI",C24="SÍ",C24=TRUE),"✅ Aprobada",IF(OR(B24="SI",B24="SÍ",B24=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>HISTORIA DE LA FILOSOFIA MEDIEVAL</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>3° Año</t>
+        </is>
+      </c>
+      <c r="E25" s="9">
+        <f>IF(OR(B25="SI",B25="SÍ",B25=TRUE),"REGULAR","PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F25" s="9">
+        <f>IF(OR(C25="SI",C25="SÍ",C25=TRUE),"APROBADA",IF(OR(B25="SI",B25="SÍ",B25=TRUE),"RINDE FINAL","ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G25" s="9">
+        <f>IF(OR(C25="SI",C25="SÍ",C25=TRUE),"✅ Aprobada",IF(OR(B25="SI",B25="SÍ",B25=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Lógica 2</t>
+          <t>LOGICA II (1° Cuat.)</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -1413,28 +1401,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D26" s="16" t="inlineStr">
-        <is>
-          <t>Lógica 1 y Teoría de la Argumentación</t>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E26" s="9">
-        <f>IF(OR(B26="SI",B26="SÍ",B26=TRUE),"CURSADA REGULAR",IF(AND(OR(B5="SI",B5="SÍ",B5=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B26="SI",B26="SÍ",B26=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F26" s="9">
-        <f>IF(OR(C26="SI",C26="SÍ",C26=TRUE),"APROBADA",IF(AND(OR(B26="SI",B26="SÍ",B26=TRUE),AND(OR(C5="SI",C5="SÍ",C5=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C26="SI",C26="SÍ",C26=TRUE),"APROBADA",IF(OR(B26="SI",B26="SÍ",B26=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G26" s="9">
-        <f>IF(OR(C26="SI",C26="SÍ",C26=TRUE),"✅ Materia Aprobada",IF(OR(B26="SI",B26="SÍ",B26=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C26="SI",C26="SÍ",C26=TRUE),"✅ Aprobada",IF(OR(B26="SI",B26="SÍ",B26=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Filosofía de la Lógica</t>
+          <t>METAFISICA</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
@@ -1447,28 +1435,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
-        <is>
-          <t>Lógica 1 y Teoría de la Argumentación</t>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E27" s="9">
-        <f>IF(OR(B27="SI",B27="SÍ",B27=TRUE),"CURSADA REGULAR",IF(AND(OR(B5="SI",B5="SÍ",B5=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B27="SI",B27="SÍ",B27=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F27" s="9">
-        <f>IF(OR(C27="SI",C27="SÍ",C27=TRUE),"APROBADA",IF(AND(OR(B27="SI",B27="SÍ",B27=TRUE),AND(OR(C5="SI",C5="SÍ",C5=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C27="SI",C27="SÍ",C27=TRUE),"APROBADA",IF(OR(B27="SI",B27="SÍ",B27=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G27" s="9">
-        <f>IF(OR(C27="SI",C27="SÍ",C27=TRUE),"✅ Materia Aprobada",IF(OR(B27="SI",B27="SÍ",B27=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C27="SI",C27="SÍ",C27=TRUE),"✅ Aprobada",IF(OR(B27="SI",B27="SÍ",B27=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Historia de la Filosofía Medieval</t>
+          <t>SISTEMA Y POLITICA EDUCATIVA (1° CUATR.)</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -1481,28 +1469,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Antigua</t>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E28" s="9">
-        <f>IF(OR(B28="SI",B28="SÍ",B28=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B28="SI",B28="SÍ",B28=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F28" s="9">
-        <f>IF(OR(C28="SI",C28="SÍ",C28=TRUE),"APROBADA",IF(AND(OR(B28="SI",B28="SÍ",B28=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C28="SI",C28="SÍ",C28=TRUE),"APROBADA",IF(OR(B28="SI",B28="SÍ",B28=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G28" s="9">
-        <f>IF(OR(C28="SI",C28="SÍ",C28=TRUE),"✅ Materia Aprobada",IF(OR(B28="SI",B28="SÍ",B28=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C28="SI",C28="SÍ",C28=TRUE),"✅ Aprobada",IF(OR(B28="SI",B28="SÍ",B28=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Metafísica</t>
+          <t>TALLER DIDACT.DE LA FILO Y PROD.MAT.ED</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1515,28 +1503,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Antigua</t>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E29" s="9">
-        <f>IF(OR(B29="SI",B29="SÍ",B29=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B29="SI",B29="SÍ",B29=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F29" s="9">
-        <f>IF(OR(C29="SI",C29="SÍ",C29=TRUE),"APROBADA",IF(AND(OR(B29="SI",B29="SÍ",B29=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C29="SI",C29="SÍ",C29=TRUE),"APROBADA",IF(OR(B29="SI",B29="SÍ",B29=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G29" s="9">
-        <f>IF(OR(C29="SI",C29="SÍ",C29=TRUE),"✅ Materia Aprobada",IF(OR(B29="SI",B29="SÍ",B29=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C29="SI",C29="SÍ",C29=TRUE),"✅ Aprobada",IF(OR(B29="SI",B29="SÍ",B29=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Historia de la Ciencia</t>
+          <t>TALLER FILOSOFIA Y EDUCACION</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -1549,28 +1537,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>Metodología de la Investigación</t>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E30" s="9">
-        <f>IF(OR(B30="SI",B30="SÍ",B30=TRUE),"CURSADA REGULAR",IF(AND(OR(B21="SI",B21="SÍ",B21=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B30="SI",B30="SÍ",B30=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F30" s="9">
-        <f>IF(OR(C30="SI",C30="SÍ",C30=TRUE),"APROBADA",IF(AND(OR(B30="SI",B30="SÍ",B30=TRUE),AND(OR(C21="SI",C21="SÍ",C21=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C30="SI",C30="SÍ",C30=TRUE),"APROBADA",IF(OR(B30="SI",B30="SÍ",B30=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G30" s="9">
-        <f>IF(OR(C30="SI",C30="SÍ",C30=TRUE),"✅ Materia Aprobada",IF(OR(B30="SI",B30="SÍ",B30=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C30="SI",C30="SÍ",C30=TRUE),"✅ Aprobada",IF(OR(B30="SI",B30="SÍ",B30=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Trabajo de Campo 3</t>
+          <t>TEORIA DEL CONOCIMIENTO</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -1583,28 +1571,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
-        <is>
-          <t>Trabajo de Campo 2</t>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E31" s="9">
-        <f>IF(OR(B31="SI",B31="SÍ",B31=TRUE),"CURSADA REGULAR",IF(AND(OR(B24="SI",B24="SÍ",B24=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B31="SI",B31="SÍ",B31=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F31" s="9">
-        <f>IF(OR(C31="SI",C31="SÍ",C31=TRUE),"APROBADA",IF(AND(OR(B31="SI",B31="SÍ",B31=TRUE),AND(OR(C24="SI",C24="SÍ",C24=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C31="SI",C31="SÍ",C31=TRUE),"APROBADA",IF(OR(B31="SI",B31="SÍ",B31=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G31" s="9">
-        <f>IF(OR(C31="SI",C31="SÍ",C31=TRUE),"✅ Materia Aprobada",IF(OR(B31="SI",B31="SÍ",B31=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C31="SI",C31="SÍ",C31=TRUE),"✅ Aprobada",IF(OR(B31="SI",B31="SÍ",B31=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Taller de Didáctica de la Filosofía y Prod. Materiales</t>
+          <t>TRABAJO DE CAMPO III</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -1617,62 +1605,35 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>Didáctica General</t>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E32" s="9">
-        <f>IF(OR(B32="SI",B32="SÍ",B32=TRUE),"CURSADA REGULAR",IF(AND(OR(B16="SI",B16="SÍ",B16=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B32="SI",B32="SÍ",B32=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F32" s="9">
-        <f>IF(OR(C32="SI",C32="SÍ",C32=TRUE),"APROBADA",IF(AND(OR(B32="SI",B32="SÍ",B32=TRUE),AND(OR(C16="SI",C16="SÍ",C16=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C32="SI",C32="SÍ",C32=TRUE),"APROBADA",IF(OR(B32="SI",B32="SÍ",B32=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G32" s="9">
-        <f>IF(OR(C32="SI",C32="SÍ",C32=TRUE),"✅ Materia Aprobada",IF(OR(B32="SI",B32="SÍ",B32=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>Sistema y Política Educativa</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>Historia de la Educación Argentina</t>
-        </is>
-      </c>
-      <c r="E33" s="9">
-        <f>IF(OR(B33="SI",B33="SÍ",B33=TRUE),"CURSADA REGULAR",IF(AND(OR(B17="SI",B17="SÍ",B17=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
-        <v/>
-      </c>
-      <c r="F33" s="9">
-        <f>IF(OR(C33="SI",C33="SÍ",C33=TRUE),"APROBADA",IF(AND(OR(B33="SI",B33="SÍ",B33=TRUE),AND(OR(C17="SI",C17="SÍ",C17=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
-        <v/>
-      </c>
-      <c r="G33" s="9">
-        <f>IF(OR(C33="SI",C33="SÍ",C33=TRUE),"✅ Materia Aprobada",IF(OR(B33="SI",B33="SÍ",B33=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
+        <f>IF(OR(C32="SI",C32="SÍ",C32=TRUE),"✅ Aprobada",IF(OR(B32="SI",B32="SÍ",B32=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>📌 4° AÑO</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Taller Filosofía y Educación</t>
+          <t>ESTETICA</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -1685,28 +1646,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Antigua</t>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E34" s="9">
-        <f>IF(OR(B34="SI",B34="SÍ",B34=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B34="SI",B34="SÍ",B34=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F34" s="9">
-        <f>IF(OR(C34="SI",C34="SÍ",C34=TRUE),"APROBADA",IF(AND(OR(B34="SI",B34="SÍ",B34=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C34="SI",C34="SÍ",C34=TRUE),"APROBADA",IF(OR(B34="SI",B34="SÍ",B34=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G34" s="9">
-        <f>IF(OR(C34="SI",C34="SÍ",C34=TRUE),"✅ Materia Aprobada",IF(OR(B34="SI",B34="SÍ",B34=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C34="SI",C34="SÍ",C34=TRUE),"✅ Aprobada",IF(OR(B34="SI",B34="SÍ",B34=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Teoría del Conocimiento</t>
+          <t>FILOSOFIA DEL LENGUAJE</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -1719,28 +1680,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Antigua</t>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E35" s="9">
-        <f>IF(OR(B35="SI",B35="SÍ",B35=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B35="SI",B35="SÍ",B35=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F35" s="9">
-        <f>IF(OR(C35="SI",C35="SÍ",C35=TRUE),"APROBADA",IF(AND(OR(B35="SI",B35="SÍ",B35=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C35="SI",C35="SÍ",C35=TRUE),"APROBADA",IF(OR(B35="SI",B35="SÍ",B35=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G35" s="9">
-        <f>IF(OR(C35="SI",C35="SÍ",C35=TRUE),"✅ Materia Aprobada",IF(OR(B35="SI",B35="SÍ",B35=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C35="SI",C35="SÍ",C35=TRUE),"✅ Aprobada",IF(OR(B35="SI",B35="SÍ",B35=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Ética</t>
+          <t>FILOSOFIA POLITICA</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -1753,35 +1714,62 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>Introducción a la Filosofía</t>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E36" s="9">
-        <f>IF(OR(B36="SI",B36="SÍ",B36=TRUE),"CURSADA REGULAR",IF(AND(OR(B6="SI",B6="SÍ",B6=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B36="SI",B36="SÍ",B36=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F36" s="9">
-        <f>IF(OR(C36="SI",C36="SÍ",C36=TRUE),"APROBADA",IF(AND(OR(B36="SI",B36="SÍ",B36=TRUE),AND(OR(C6="SI",C6="SÍ",C6=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C36="SI",C36="SÍ",C36=TRUE),"APROBADA",IF(OR(B36="SI",B36="SÍ",B36=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G36" s="9">
-        <f>IF(OR(C36="SI",C36="SÍ",C36=TRUE),"✅ Materia Aprobada",IF(OR(B36="SI",B36="SÍ",B36=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>📌 CUARTO AÑO</t>
-        </is>
+        <f>IF(OR(C36="SI",C36="SÍ",C36=TRUE),"✅ Aprobada",IF(OR(B36="SI",B36="SÍ",B36=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>HISTORIA DE LA FILOSOFIA MODERNA</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
+        </is>
+      </c>
+      <c r="E37" s="9">
+        <f>IF(OR(B37="SI",B37="SÍ",B37=TRUE),"REGULAR","PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F37" s="9">
+        <f>IF(OR(C37="SI",C37="SÍ",C37=TRUE),"APROBADA",IF(OR(B37="SI",B37="SÍ",B37=TRUE),"RINDE FINAL","ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G37" s="9">
+        <f>IF(OR(C37="SI",C37="SÍ",C37=TRUE),"✅ Aprobada",IF(OR(B37="SI",B37="SÍ",B37=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Historia de la Filosofía Moderna</t>
+          <t>SEMINARIO DE ANTROPOLOGÍA FILOSÓFICA "A"</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -1794,28 +1782,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D38" s="16" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Medieval</t>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E38" s="9">
-        <f>IF(OR(B38="SI",B38="SÍ",B38=TRUE),"CURSADA REGULAR",IF(AND(OR(B28="SI",B28="SÍ",B28=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B38="SI",B38="SÍ",B38=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F38" s="9">
-        <f>IF(OR(C38="SI",C38="SÍ",C38=TRUE),"APROBADA",IF(AND(OR(B38="SI",B38="SÍ",B38=TRUE),AND(OR(C28="SI",C28="SÍ",C28=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C38="SI",C38="SÍ",C38=TRUE),"APROBADA",IF(OR(B38="SI",B38="SÍ",B38=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G38" s="9">
-        <f>IF(OR(C38="SI",C38="SÍ",C38=TRUE),"✅ Materia Aprobada",IF(OR(B38="SI",B38="SÍ",B38=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C38="SI",C38="SÍ",C38=TRUE),"✅ Aprobada",IF(OR(B38="SI",B38="SÍ",B38=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Filosofía Política</t>
+          <t>SEMINARIO DE FILOSOFIA ANTIGUA Y MEDIEVAL</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -1828,62 +1816,35 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D39" s="17" t="inlineStr">
-        <is>
-          <t>Filosofía Argentina y Latinoamericana, Ética</t>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E39" s="9">
-        <f>IF(OR(B39="SI",B39="SÍ",B39=TRUE),"CURSADA REGULAR",IF(AND(OR(B19="SI",B19="SÍ",B19=TRUE),OR(B36="SI",B36="SÍ",B36=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B39="SI",B39="SÍ",B39=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F39" s="9">
-        <f>IF(OR(C39="SI",C39="SÍ",C39=TRUE),"APROBADA",IF(AND(OR(B39="SI",B39="SÍ",B39=TRUE),AND(OR(C19="SI",C19="SÍ",C19=TRUE),OR(C36="SI",C36="SÍ",C36=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C39="SI",C39="SÍ",C39=TRUE),"APROBADA",IF(OR(B39="SI",B39="SÍ",B39=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G39" s="9">
-        <f>IF(OR(C39="SI",C39="SÍ",C39=TRUE),"✅ Materia Aprobada",IF(OR(B39="SI",B39="SÍ",B39=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>Filosofía del Lenguaje</t>
-        </is>
-      </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
-        <is>
-          <t>Filosofía de la Lógica</t>
-        </is>
-      </c>
-      <c r="E40" s="9">
-        <f>IF(OR(B40="SI",B40="SÍ",B40=TRUE),"CURSADA REGULAR",IF(AND(OR(B27="SI",B27="SÍ",B27=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
-        <v/>
-      </c>
-      <c r="F40" s="9">
-        <f>IF(OR(C40="SI",C40="SÍ",C40=TRUE),"APROBADA",IF(AND(OR(B40="SI",B40="SÍ",B40=TRUE),AND(OR(C27="SI",C27="SÍ",C27=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
-        <v/>
-      </c>
-      <c r="G40" s="9">
-        <f>IF(OR(C40="SI",C40="SÍ",C40=TRUE),"✅ Materia Aprobada",IF(OR(B40="SI",B40="SÍ",B40=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
+        <f>IF(OR(C39="SI",C39="SÍ",C39=TRUE),"✅ Aprobada",IF(OR(B39="SI",B39="SÍ",B39=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>📌 5° AÑO (NIVEL SUPERIOR / TRAMO SUPERIOR)</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Antropología Filosófica</t>
+          <t>ANTROPOLOGIA CULTURAL (OPTATIVA I)</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -1896,28 +1857,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D41" s="17" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Antigua</t>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
       <c r="E41" s="9">
-        <f>IF(OR(B41="SI",B41="SÍ",B41=TRUE),"CURSADA REGULAR",IF(AND(OR(B18="SI",B18="SÍ",B18=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B41="SI",B41="SÍ",B41=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F41" s="9">
-        <f>IF(OR(C41="SI",C41="SÍ",C41=TRUE),"APROBADA",IF(AND(OR(B41="SI",B41="SÍ",B41=TRUE),AND(OR(C18="SI",C18="SÍ",C18=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C41="SI",C41="SÍ",C41=TRUE),"APROBADA",IF(OR(B41="SI",B41="SÍ",B41=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G41" s="9">
-        <f>IF(OR(C41="SI",C41="SÍ",C41=TRUE),"✅ Materia Aprobada",IF(OR(B41="SI",B41="SÍ",B41=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C41="SI",C41="SÍ",C41=TRUE),"✅ Aprobada",IF(OR(B41="SI",B41="SÍ",B41=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Estética</t>
+          <t>FILOSOFIA CONTEMPORANEA</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
@@ -1930,28 +1891,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>Historia del Arte</t>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
       <c r="E42" s="9">
-        <f>IF(OR(B42="SI",B42="SÍ",B42=TRUE),"CURSADA REGULAR",IF(AND(OR(B20="SI",B20="SÍ",B20=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B42="SI",B42="SÍ",B42=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F42" s="9">
-        <f>IF(OR(C42="SI",C42="SÍ",C42=TRUE),"APROBADA",IF(AND(OR(B42="SI",B42="SÍ",B42=TRUE),AND(OR(C20="SI",C20="SÍ",C20=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C42="SI",C42="SÍ",C42=TRUE),"APROBADA",IF(OR(B42="SI",B42="SÍ",B42=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G42" s="9">
-        <f>IF(OR(C42="SI",C42="SÍ",C42=TRUE),"✅ Materia Aprobada",IF(OR(B42="SI",B42="SÍ",B42=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C42="SI",C42="SÍ",C42=TRUE),"✅ Aprobada",IF(OR(B42="SI",B42="SÍ",B42=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Práctica Docente 1</t>
+          <t>FILOSOFIA DE GENERO (OPTATIVA II)</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -1964,35 +1925,62 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
-        <is>
-          <t>Taller de Didáctica de la Filosofía y Prod. Materiales, Trabajo de Campo 3</t>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
       <c r="E43" s="9">
-        <f>IF(OR(B43="SI",B43="SÍ",B43=TRUE),"CURSADA REGULAR",IF(AND(OR(B32="SI",B32="SÍ",B32=TRUE),OR(B31="SI",B31="SÍ",B31=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B43="SI",B43="SÍ",B43=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F43" s="9">
-        <f>IF(OR(C43="SI",C43="SÍ",C43=TRUE),"APROBADA",IF(AND(OR(B43="SI",B43="SÍ",B43=TRUE),AND(OR(C32="SI",C32="SÍ",C32=TRUE),OR(C31="SI",C31="SÍ",C31=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C43="SI",C43="SÍ",C43=TRUE),"APROBADA",IF(OR(B43="SI",B43="SÍ",B43=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G43" s="9">
-        <f>IF(OR(C43="SI",C43="SÍ",C43=TRUE),"✅ Materia Aprobada",IF(OR(B43="SI",B43="SÍ",B43=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="24" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>📌 QUINTO AÑO</t>
-        </is>
+        <f>IF(OR(C43="SI",C43="SÍ",C43=TRUE),"✅ Aprobada",IF(OR(B43="SI",B43="SÍ",B43=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>FILOSOFIA DE LA CIENCIA</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
+        </is>
+      </c>
+      <c r="E44" s="9">
+        <f>IF(OR(B44="SI",B44="SÍ",B44=TRUE),"REGULAR","PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F44" s="9">
+        <f>IF(OR(C44="SI",C44="SÍ",C44=TRUE),"APROBADA",IF(OR(B44="SI",B44="SÍ",B44=TRUE),"RINDE FINAL","ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G44" s="9">
+        <f>IF(OR(C44="SI",C44="SÍ",C44=TRUE),"✅ Aprobada",IF(OR(B44="SI",B44="SÍ",B44=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Historia de la Filosofía Contemporánea</t>
+          <t>FILOSOFIA DE LA HISTORIA</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
@@ -2005,28 +1993,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D45" s="17" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Moderna</t>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
       <c r="E45" s="9">
-        <f>IF(OR(B45="SI",B45="SÍ",B45=TRUE),"CURSADA REGULAR",IF(AND(OR(B38="SI",B38="SÍ",B38=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B45="SI",B45="SÍ",B45=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F45" s="9">
-        <f>IF(OR(C45="SI",C45="SÍ",C45=TRUE),"APROBADA",IF(AND(OR(B45="SI",B45="SÍ",B45=TRUE),AND(OR(C38="SI",C38="SÍ",C38=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C45="SI",C45="SÍ",C45=TRUE),"APROBADA",IF(OR(B45="SI",B45="SÍ",B45=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G45" s="9">
-        <f>IF(OR(C45="SI",C45="SÍ",C45=TRUE),"✅ Materia Aprobada",IF(OR(B45="SI",B45="SÍ",B45=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C45="SI",C45="SÍ",C45=TRUE),"✅ Aprobada",IF(OR(B45="SI",B45="SÍ",B45=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>Filosofía del Derecho</t>
+          <t>FILOSOFIA DE LA RELIGION</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
@@ -2039,28 +2027,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>Filosofía Política</t>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
       <c r="E46" s="9">
-        <f>IF(OR(B46="SI",B46="SÍ",B46=TRUE),"CURSADA REGULAR",IF(AND(OR(B39="SI",B39="SÍ",B39=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B46="SI",B46="SÍ",B46=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F46" s="9">
-        <f>IF(OR(C46="SI",C46="SÍ",C46=TRUE),"APROBADA",IF(AND(OR(B46="SI",B46="SÍ",B46=TRUE),AND(OR(C39="SI",C39="SÍ",C39=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C46="SI",C46="SÍ",C46=TRUE),"APROBADA",IF(OR(B46="SI",B46="SÍ",B46=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G46" s="9">
-        <f>IF(OR(C46="SI",C46="SÍ",C46=TRUE),"✅ Materia Aprobada",IF(OR(B46="SI",B46="SÍ",B46=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C46="SI",C46="SÍ",C46=TRUE),"✅ Aprobada",IF(OR(B46="SI",B46="SÍ",B46=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>Filosofía de la Religión</t>
+          <t>RESIDENCIA</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -2073,28 +2061,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D47" s="17" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Medieval</t>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
       <c r="E47" s="9">
-        <f>IF(OR(B47="SI",B47="SÍ",B47=TRUE),"CURSADA REGULAR",IF(AND(OR(B28="SI",B28="SÍ",B28=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B47="SI",B47="SÍ",B47=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F47" s="9">
-        <f>IF(OR(C47="SI",C47="SÍ",C47=TRUE),"APROBADA",IF(AND(OR(B47="SI",B47="SÍ",B47=TRUE),AND(OR(C28="SI",C28="SÍ",C28=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C47="SI",C47="SÍ",C47=TRUE),"APROBADA",IF(OR(B47="SI",B47="SÍ",B47=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G47" s="9">
-        <f>IF(OR(C47="SI",C47="SÍ",C47=TRUE),"✅ Materia Aprobada",IF(OR(B47="SI",B47="SÍ",B47=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C47="SI",C47="SÍ",C47=TRUE),"✅ Aprobada",IF(OR(B47="SI",B47="SÍ",B47=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>Filosofía de la Historia</t>
+          <t>SEMINARIO DE FILOSOFIA MODERNA Y CONTEMPORANEA</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
@@ -2107,28 +2095,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>Historia de la Filosofía Moderna</t>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
       <c r="E48" s="9">
-        <f>IF(OR(B48="SI",B48="SÍ",B48=TRUE),"CURSADA REGULAR",IF(AND(OR(B38="SI",B38="SÍ",B38=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B48="SI",B48="SÍ",B48=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F48" s="9">
-        <f>IF(OR(C48="SI",C48="SÍ",C48=TRUE),"APROBADA",IF(AND(OR(B48="SI",B48="SÍ",B48=TRUE),AND(OR(C38="SI",C38="SÍ",C38=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C48="SI",C48="SÍ",C48=TRUE),"APROBADA",IF(OR(B48="SI",B48="SÍ",B48=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G48" s="9">
-        <f>IF(OR(C48="SI",C48="SÍ",C48=TRUE),"✅ Materia Aprobada",IF(OR(B48="SI",B48="SÍ",B48=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C48="SI",C48="SÍ",C48=TRUE),"✅ Aprobada",IF(OR(B48="SI",B48="SÍ",B48=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>Filosofía de la Ciencia</t>
+          <t>SOCIEDAD, ESTADO Y DD HH</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -2141,78 +2129,188 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D49" s="17" t="inlineStr">
-        <is>
-          <t>Historia de la Ciencia, Teoría del Conocimiento</t>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
       <c r="E49" s="9">
-        <f>IF(OR(B49="SI",B49="SÍ",B49=TRUE),"CURSADA REGULAR",IF(AND(OR(B30="SI",B30="SÍ",B30=TRUE),OR(B35="SI",B35="SÍ",B35=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
+        <f>IF(OR(B49="SI",B49="SÍ",B49=TRUE),"REGULAR","PENDIENTE")</f>
         <v/>
       </c>
       <c r="F49" s="9">
-        <f>IF(OR(C49="SI",C49="SÍ",C49=TRUE),"APROBADA",IF(AND(OR(B49="SI",B49="SÍ",B49=TRUE),AND(OR(C30="SI",C30="SÍ",C30=TRUE),OR(C35="SI",C35="SÍ",C35=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
+        <f>IF(OR(C49="SI",C49="SÍ",C49=TRUE),"APROBADA",IF(OR(B49="SI",B49="SÍ",B49=TRUE),"RINDE FINAL","ADEUDA"))</f>
         <v/>
       </c>
       <c r="G49" s="9">
-        <f>IF(OR(C49="SI",C49="SÍ",C49=TRUE),"✅ Materia Aprobada",IF(OR(B49="SI",B49="SÍ",B49=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="11" t="inlineStr">
-        <is>
-          <t>Práctica Docente 2 y Residencia</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>Práctica Docente 1</t>
-        </is>
-      </c>
-      <c r="E50" s="9">
-        <f>IF(OR(B50="SI",B50="SÍ",B50=TRUE),"CURSADA REGULAR",IF(AND(OR(B43="SI",B43="SÍ",B43=TRUE)),"¡HABILITADA!","Faltan correlat."))</f>
-        <v/>
-      </c>
-      <c r="F50" s="9">
-        <f>IF(OR(C50="SI",C50="SÍ",C50=TRUE),"APROBADA",IF(AND(OR(B50="SI",B50="SÍ",B50=TRUE),AND(OR(C43="SI",C43="SÍ",C43=TRUE))),"¡LISTO P/ FINAL!","Faltan finales prev."))</f>
-        <v/>
-      </c>
-      <c r="G50" s="9">
-        <f>IF(OR(C50="SI",C50="SÍ",C50=TRUE),"✅ Materia Aprobada",IF(OR(B50="SI",B50="SÍ",B50=TRUE),"⏳ Regular (Adeuda Final)","⚪ Pendiente"))</f>
+        <f>IF(OR(C49="SI",C49="SÍ",C49=TRUE),"✅ Aprobada",IF(OR(B49="SI",B49="SÍ",B49=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>📌 6° AÑO (NIVEL SUPERIOR / TRAMO SUPERIOR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Seminario de Especialización Superior II</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>6° Año (Nivel Superior / Tramo Superior)</t>
+        </is>
+      </c>
+      <c r="E51" s="9">
+        <f>IF(OR(B51="SI",B51="SÍ",B51=TRUE),"REGULAR","PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F51" s="9">
+        <f>IF(OR(C51="SI",C51="SÍ",C51=TRUE),"APROBADA",IF(OR(B51="SI",B51="SÍ",B51=TRUE),"RINDE FINAL","ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G51" s="9">
+        <f>IF(OR(C51="SI",C51="SÍ",C51=TRUE),"✅ Aprobada",IF(OR(B51="SI",B51="SÍ",B51=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>Tesis / Trabajo Final de Licenciatura</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>6° Año (Nivel Superior / Tramo Superior)</t>
+        </is>
+      </c>
+      <c r="E52" s="9">
+        <f>IF(OR(B52="SI",B52="SÍ",B52=TRUE),"REGULAR","PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F52" s="9">
+        <f>IF(OR(C52="SI",C52="SÍ",C52=TRUE),"APROBADA",IF(OR(B52="SI",B52="SÍ",B52=TRUE),"RINDE FINAL","ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G52" s="9">
+        <f>IF(OR(C52="SI",C52="SÍ",C52=TRUE),"✅ Aprobada",IF(OR(B52="SI",B52="SÍ",B52=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>Práctica de Nivel Superior II</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>6° Año (Nivel Superior / Tramo Superior)</t>
+        </is>
+      </c>
+      <c r="E53" s="9">
+        <f>IF(OR(B53="SI",B53="SÍ",B53=TRUE),"REGULAR","PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F53" s="9">
+        <f>IF(OR(C53="SI",C53="SÍ",C53=TRUE),"APROBADA",IF(OR(B53="SI",B53="SÍ",B53=TRUE),"RINDE FINAL","ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G53" s="9">
+        <f>IF(OR(C53="SI",C53="SÍ",C53=TRUE),"✅ Aprobada",IF(OR(B53="SI",B53="SÍ",B53=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>Acreditación de Residencia Superior</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>6° Año (Nivel Superior / Tramo Superior)</t>
+        </is>
+      </c>
+      <c r="E54" s="9">
+        <f>IF(OR(B54="SI",B54="SÍ",B54=TRUE),"REGULAR","PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F54" s="9">
+        <f>IF(OR(C54="SI",C54="SÍ",C54=TRUE),"APROBADA",IF(OR(B54="SI",B54="SÍ",B54=TRUE),"RINDE FINAL","ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G54" s="9">
+        <f>IF(OR(C54="SI",C54="SÍ",C54=TRUE),"✅ Aprobada",IF(OR(B54="SI",B54="SÍ",B54=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="A44:G44"/>
+  <mergeCells count="16">
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I3:J3"/>
     <mergeCell ref="I15:J15"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A50:G50"/>
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:G15"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="A33:G33"/>
     <mergeCell ref="I17:J17"/>
-    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="I3:J3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B5:C50" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B4:C54" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>